<commit_message>
Spellcheck: fix "Begining" -> "Beginning" in category names, correct stale instruction wording
The teacher-instructions line about marking incorrect words referenced
"the three words", left over from when categories were always exactly
3 words - most aren't. Reworded to be category-agnostic.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DZEHcZ6zSYn9tyL9u8ex4z
</commit_message>
<xml_diff>
--- a/data/source/Ganeinu_Assessments_for_Kriah_Curriculum.xlsx
+++ b/data/source/Ganeinu_Assessments_for_Kriah_Curriculum.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="H2" t="str" xml:space="preserve">
         <v xml:space="preserve">Sheva in _x000d_
-Begining </v>
+Beginning </v>
       </c>
       <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">Sheva in _x000d_
@@ -471,7 +471,7 @@
       </c>
       <c r="Q2" t="str" xml:space="preserve">
         <v xml:space="preserve">Shuruk in _x000d_
-begining</v>
+beginning</v>
       </c>
       <c r="R2" t="str" xml:space="preserve">
         <v xml:space="preserve">Confusing Dagesh_x000d_

</xml_diff>

<commit_message>
Spellcheck: fix "Begining" -> "Beginning" in category names, correct stale instruction wording (#12)
The teacher-instructions line about marking incorrect words referenced
"the three words", left over from when categories were always exactly
3 words - most aren't. Reworded to be category-agnostic.


Claude-Session: https://claude.ai/code/session_01DZEHcZ6zSYn9tyL9u8ex4z

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Ganeinu_Assessments_for_Kriah_Curriculum.xlsx
+++ b/data/source/Ganeinu_Assessments_for_Kriah_Curriculum.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="H2" t="str" xml:space="preserve">
         <v xml:space="preserve">Sheva in _x000d_
-Begining </v>
+Beginning </v>
       </c>
       <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">Sheva in _x000d_
@@ -471,7 +471,7 @@
       </c>
       <c r="Q2" t="str" xml:space="preserve">
         <v xml:space="preserve">Shuruk in _x000d_
-begining</v>
+beginning</v>
       </c>
       <c r="R2" t="str" xml:space="preserve">
         <v xml:space="preserve">Confusing Dagesh_x000d_

</xml_diff>